<commit_message>
Added some parts into excel & added cad file for project concept
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F2943F1-C3D6-4C7D-9241-1387F743205B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E404C5A-17AB-4F01-B16E-6AC5D0794B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Bills Of Material" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>No.</t>
   </si>
@@ -66,13 +66,28 @@
   </si>
   <si>
     <t>Marble Station with ESP32</t>
+  </si>
+  <si>
+    <t>Servo Motor</t>
+  </si>
+  <si>
+    <t>Servo Motor 180</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1o-F_MPZrxvgcB_fcxiyyhbE7Jak8m61UF-xSTBCvfaY/edit?gid=2086349135#gid=2086349135</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,6 +121,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -292,17 +315,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -312,6 +333,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -327,31 +354,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -369,14 +395,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor rgb="FFC00000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -710,92 +729,125 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5785CA-F4AE-4464-AE2C-5F7A426F62CB}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="42.375" customWidth="1"/>
+    <col min="2" max="2" width="42.42578125" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
-    <col min="5" max="5" width="25.5" customWidth="1"/>
-    <col min="6" max="6" width="17.875" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="12" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="9"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12"/>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="11"/>
     </row>
-    <row r="3" spans="1:6" ht="15">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="16">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="15">
+        <v>3</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="16">
+        <v>2</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="17" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"In Stock"</formula>
+  <conditionalFormatting sqref="G4:G5">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Not ordered"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Ordered"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Not ordered"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"In Stock"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G5" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E4" r:id="rId1" location="gid=2086349135" xr:uid="{D19C5093-5F1E-43F6-A2F5-6AD80406CC4D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added draft (ESP32 blinking test)
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E404C5A-17AB-4F01-B16E-6AC5D0794B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48181BF-D7D5-4210-9D29-7B3FEE1217A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
+    <workbookView xWindow="7305" yWindow="3045" windowWidth="24045" windowHeight="15930" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="Bills Of Material" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>No.</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>ESP32-C3 Supermini</t>
-  </si>
-  <si>
     <t>Main controller (Wi-Fi + Bluetooth)</t>
   </si>
   <si>
@@ -77,7 +74,31 @@
     <t>Link</t>
   </si>
   <si>
-    <t>https://docs.google.com/spreadsheets/d/1o-F_MPZrxvgcB_fcxiyyhbE7Jak8m61UF-xSTBCvfaY/edit?gid=2086349135#gid=2086349135</t>
+    <t>USB-C Cable</t>
+  </si>
+  <si>
+    <t>USB-C Cable 3m</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/ANMIEL-Typ-C-Kabel-Ladekabel-Datenkabel-geflochten/dp/B09C3HH7KJ/ref=sr_1_6?__mk_de_DE=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=1HUJ8X6PSQNU8&amp;dib=eyJ2IjoiMSJ9.ZH0eL8XvX3DTxCgYcgGTokPY-OCGP9OmCfUbJRX_O8dVp8Y1XLwoEsrPFcvnPVLZvmFR-zCeVbO2opkI9v6wstHb3PzAZOQLPOyeihnSe59NsRuwoXQmF8VlHnoIDHRuSmQaxgReVVoqtUnIHtv6TfrKTgO9Kh6iiAGngLh5Ulc8iYjsqR6B1GuoUGYiygCZirhfQUZHJkvbFNL__RF-xSf5BIU2C9X4cmz_-YjN3Lo.3DULeIhGb1u3SODSffwhRyhMYPrRy90LZrRDQ7fSg-g&amp;dib_tag=se&amp;keywords=usb%2Bc%2Bkabel%2Bdata%2B3m&amp;qid=1761953154&amp;sprefix=usb%2Bc%2Bkabel%2Bdata%2B3m%2Caps%2C103&amp;sr=8-6&amp;th=1</t>
+  </si>
+  <si>
+    <t>Not ordered</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Cable</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>Cable for slaves (up to 25m)</t>
+  </si>
+  <si>
+    <t>ESP-WROOM-32 ESP32-S</t>
   </si>
 </sst>
 </file>
@@ -85,9 +106,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,6 +150,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -319,7 +346,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -336,41 +363,45 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="6" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -729,35 +760,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5785CA-F4AE-4464-AE2C-5F7A426F62CB}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.42578125" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
-    <col min="5" max="5" width="31.140625" style="12" customWidth="1"/>
-    <col min="6" max="6" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" style="11" customWidth="1"/>
     <col min="7" max="7" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="8"/>
+      <c r="A1" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="11"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -773,10 +804,10 @@
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>7</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>4</v>
@@ -786,49 +817,96 @@
       <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="7">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="16">
-        <v>1</v>
-      </c>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="10">
+        <v>3</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>6</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="15">
-        <v>3</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="16">
-        <v>2</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="17" t="s">
-        <v>7</v>
+      <c r="E5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="7">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="10">
+        <v>8.15</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="7">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G4:G5">
+  <phoneticPr fontId="6" type="noConversion"/>
+  <conditionalFormatting sqref="G4:G7">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Not ordered"</formula>
     </cfRule>
@@ -840,14 +918,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G5" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G7" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" location="gid=2086349135" xr:uid="{D19C5093-5F1E-43F6-A2F5-6AD80406CC4D}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished PCB Power Jack
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A43CF9-DDF2-493D-8D59-10072326EF2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A4EBF8C-E846-4019-8126-162ECD6E215D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="46">
   <si>
     <t>No.</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Marble Station with ESP32</t>
   </si>
   <si>
-    <t>Link</t>
-  </si>
-  <si>
     <t>USB-C Cable</t>
   </si>
   <si>
@@ -134,12 +131,6 @@
     <t>122 Stück Elektrolytkondensator 16 V 25 V 50 V Aluminium</t>
   </si>
   <si>
-    <t>Small Fuse</t>
-  </si>
-  <si>
-    <t>Small Fuse &amp; Holder 3A 5 Set</t>
-  </si>
-  <si>
     <t>Power Jack Port</t>
   </si>
   <si>
@@ -162,6 +153,27 @@
   </si>
   <si>
     <t>Gravi Tax Base</t>
+  </si>
+  <si>
+    <t>PCB Production</t>
+  </si>
+  <si>
+    <t>Jack Power PCB</t>
+  </si>
+  <si>
+    <t>JLCPcb</t>
+  </si>
+  <si>
+    <t>Ordered</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>SMD Electrolytic Cap.</t>
+  </si>
+  <si>
+    <t>16V 1000uF 10x10.2</t>
   </si>
 </sst>
 </file>
@@ -235,13 +247,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -460,6 +472,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -478,18 +505,6 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -501,9 +516,6 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -862,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5785CA-F4AE-4464-AE2C-5F7A426F62CB}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.42578125" customWidth="1"/>
@@ -873,24 +885,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="21"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="19"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -906,7 +918,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>6</v>
@@ -920,7 +932,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -929,13 +941,13 @@
         <v>5</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F4" s="10">
         <v>4.49</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -943,46 +955,46 @@
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="10">
         <f>C5 * 3.69</f>
         <v>7.38</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="25">
         <v>3</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="26">
+        <v>1</v>
+      </c>
+      <c r="D6" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="21">
-        <v>1</v>
-      </c>
-      <c r="D6" s="21" t="s">
+      <c r="E6" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="23">
+      <c r="F6" s="28">
         <v>8.15</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -990,22 +1002,22 @@
         <v>4</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="7">
         <v>1</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="10">
         <v>1.89</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1013,23 +1025,23 @@
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="7">
         <v>1</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F8" s="10">
         <f>C8 * 8.29</f>
         <v>8.2899999999999991</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1037,67 +1049,67 @@
         <v>6</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="10">
         <f>C9 * 2.47</f>
         <v>4.9400000000000004</v>
       </c>
       <c r="G9" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>7</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="15">
+        <v>1</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="17">
+        <v>250</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>8</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="15">
+        <v>1</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="24">
-        <v>7</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="25">
-        <v>1</v>
-      </c>
-      <c r="D10" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="27">
-        <v>250</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="24">
-        <v>8</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="25">
-        <v>1</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="27"/>
+      <c r="F11" s="17"/>
       <c r="G11" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1105,22 +1117,22 @@
         <v>9</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F12" s="10">
         <v>3.7</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1128,23 +1140,23 @@
         <v>10</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" s="7">
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F13" s="10">
         <f>C13 * 2.89</f>
         <v>5.78</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1152,22 +1164,22 @@
         <v>11</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C14" s="7">
-        <v>1</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>33</v>
+        <v>3</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>40</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="F14" s="10">
-        <v>1.69</v>
+        <v>9.5500000000000007</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1175,22 +1187,22 @@
         <v>12</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C15" s="7">
         <v>1</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F15" s="10">
         <v>1.35</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1198,22 +1210,22 @@
         <v>13</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" s="7">
         <v>1</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F16" s="10">
         <v>3.69</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1221,22 +1233,22 @@
         <v>14</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C17" s="7">
         <v>1</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F17" s="10">
         <v>1.94</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1244,22 +1256,22 @@
         <v>15</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C18" s="7">
         <v>1</v>
       </c>
-      <c r="D18" s="28" t="s">
-        <v>39</v>
+      <c r="D18" s="18" t="s">
+        <v>36</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F18" s="10">
         <v>1.69</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1267,22 +1279,45 @@
         <v>16</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C19" s="7">
         <v>2</v>
       </c>
-      <c r="D19" s="28" t="s">
-        <v>41</v>
+      <c r="D19" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="F19" s="10">
+        <v>1.99</v>
       </c>
       <c r="G19" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>17</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="7">
+        <v>3</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="13" t="s">
         <v>12</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1290,7 +1325,7 @@
     <mergeCell ref="A1:G2"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G19">
+  <conditionalFormatting sqref="G4:G20">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Not ordered"</formula>
     </cfRule>
@@ -1302,7 +1337,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G19" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G20" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Updated the files to the new state
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A4EBF8C-E846-4019-8126-162ECD6E215D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB1A96A-FAEC-4977-A487-752C99074440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="Bills Of Material" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="47">
   <si>
     <t>No.</t>
   </si>
@@ -113,12 +113,6 @@
     <t>3D Printer 1kg Filament</t>
   </si>
   <si>
-    <t>Adapter 5V 3A</t>
-  </si>
-  <si>
-    <t>Netzteil Adapter AC 220V DC  5V</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prototype Board </t>
   </si>
   <si>
@@ -174,6 +168,15 @@
   </si>
   <si>
     <t>16V 1000uF 10x10.2</t>
+  </si>
+  <si>
+    <t>Adapter 5V 10A</t>
+  </si>
+  <si>
+    <t>Netzteil Adapter AC 220V DC  5V 10A</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/gp/product/B0DM97JMVS/ref=sw_img_1?smid=A6FTR3WNTF6EM&amp;th=1</t>
   </si>
 </sst>
 </file>
@@ -487,6 +490,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -504,18 +519,6 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -885,24 +888,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="21"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="24"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="28"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -918,7 +921,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>6</v>
@@ -932,7 +935,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -975,22 +978,22 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="19">
         <v>3</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="20">
         <v>1</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="28">
+      <c r="F6" s="22">
         <v>8.15</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -1117,19 +1120,19 @@
         <v>9</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>17</v>
+        <v>45</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="F12" s="10">
-        <v>3.7</v>
+        <v>16.989999999999998</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>11</v>
@@ -1140,13 +1143,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C13" s="7">
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>17</v>
@@ -1164,22 +1167,22 @@
         <v>11</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14" s="7">
         <v>3</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F14" s="10">
         <v>9.5500000000000007</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1187,13 +1190,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C15" s="7">
         <v>1</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>17</v>
@@ -1210,13 +1213,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C16" s="7">
         <v>1</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>17</v>
@@ -1233,13 +1236,13 @@
         <v>14</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C17" s="7">
         <v>1</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>17</v>
@@ -1256,13 +1259,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C18" s="7">
         <v>1</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E18" s="13" t="s">
         <v>17</v>
@@ -1279,13 +1282,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C19" s="7">
         <v>2</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>17</v>
@@ -1302,13 +1305,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C20" s="7">
         <v>3</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>12</v>
@@ -1336,12 +1339,15 @@
       <formula>"In Stock"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G20" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E12" r:id="rId1" xr:uid="{E8A5AAF1-A457-44FF-B03E-B13CD56D10C7}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improved schematic, and updated excel list
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958E12CD-F6E9-4DFB-A74D-4148E3C97609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C11571-14D0-41B0-B6D0-C3EFB5CC75D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21705" yWindow="-12390" windowWidth="21810" windowHeight="18945" activeTab="1" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
+    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" activeTab="1" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Receiver" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="78">
   <si>
     <t>No.</t>
   </si>
@@ -247,6 +247,30 @@
   </si>
   <si>
     <t>Charger Module IC 50x</t>
+  </si>
+  <si>
+    <t>BSS84W-7-F</t>
+  </si>
+  <si>
+    <t>P Channel MOSFET 50V 50x</t>
+  </si>
+  <si>
+    <t>USB C Female Port</t>
+  </si>
+  <si>
+    <t>USB Type C Female Port 10x</t>
+  </si>
+  <si>
+    <t>Battery Terminal Connector</t>
+  </si>
+  <si>
+    <t>2 Pins Terminal Connector</t>
+  </si>
+  <si>
+    <t>Slide Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SK12D07 Kippschalter 3PIN </t>
   </si>
 </sst>
 </file>
@@ -1952,6 +1976,28 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="7">
+        <v>1</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="10">
+        <f>C9 * 3.89</f>
+        <v>3.89</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="J9" s="40" t="s">
         <v>50</v>
       </c>
@@ -1961,6 +2007,28 @@
       <c r="N9" s="42"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="7">
+        <v>1</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="10">
+        <f>C10 * 1.29</f>
+        <v>1.29</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="J10" s="43"/>
       <c r="K10" s="44"/>
       <c r="L10" s="44"/>
@@ -1968,6 +2036,28 @@
       <c r="N10" s="45"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="7">
+        <v>1</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="10">
+        <f>C11 * 1.77</f>
+        <v>1.77</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="J11" s="43"/>
       <c r="K11" s="44"/>
       <c r="L11" s="44"/>
@@ -1975,6 +2065,28 @@
       <c r="N11" s="45"/>
     </row>
     <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="7">
+        <v>1</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="10">
+        <f>C12 * 2.12</f>
+        <v>2.12</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="J12" s="46"/>
       <c r="K12" s="47"/>
       <c r="L12" s="47"/>
@@ -1984,7 +2096,7 @@
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J13" s="25">
         <f>SUM(F4:F30)</f>
-        <v>12.07</v>
+        <v>21.14</v>
       </c>
       <c r="K13" s="26"/>
       <c r="L13" s="26"/>
@@ -2019,7 +2131,7 @@
     <mergeCell ref="J13:N16"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G8">
+  <conditionalFormatting sqref="G4:G12">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Not ordered"</formula>
     </cfRule>
@@ -2031,7 +2143,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G8" xr:uid="{5C30DADA-6449-478F-B571-319D09B3C008}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G12" xr:uid="{5C30DADA-6449-478F-B571-319D09B3C008}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Added PCB & Library Database
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C11571-14D0-41B0-B6D0-C3EFB5CC75D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63AFBC0-4D22-4A6F-A92E-B07AB99D9DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" activeTab="1" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
+    <workbookView xWindow="-21705" yWindow="-12390" windowWidth="21810" windowHeight="18945" activeTab="1" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Receiver" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="80">
   <si>
     <t>No.</t>
   </si>
@@ -219,24 +219,12 @@
     <t>Jack Power PCB 25x</t>
   </si>
   <si>
-    <t>ESP-32 C3 Super Mini</t>
-  </si>
-  <si>
-    <t>In stock</t>
-  </si>
-  <si>
     <t>TFT 1,8 Inch RGB Display</t>
   </si>
   <si>
     <t xml:space="preserve"> Vollfarb-TFT-LCD-Anzeigemodul 128 x 160 SPI, ST7735S</t>
   </si>
   <si>
-    <t>Button</t>
-  </si>
-  <si>
-    <t>Coloured Button For directions</t>
-  </si>
-  <si>
     <t xml:space="preserve">TP4056 </t>
   </si>
   <si>
@@ -271,6 +259,24 @@
   </si>
   <si>
     <t xml:space="preserve">SK12D07 Kippschalter 3PIN </t>
+  </si>
+  <si>
+    <t>SMD-Diode SOD-123</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SMD-Diode 0805 SOD-123 S4 1N5819 100x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP-WROOM-32 </t>
+  </si>
+  <si>
+    <t>CP2102 WIFI Bluetooth-Modul Dual Core Wireless-Modul ESP-32 ESP-WROOM-32</t>
+  </si>
+  <si>
+    <t>25PCS Tactile Push Button Switch Momentary 12*12*7,3MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tacitile Push Button </t>
   </si>
 </sst>
 </file>
@@ -1860,23 +1866,23 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>17</v>
       </c>
       <c r="F4" s="10">
-        <f>C4 * 4.49</f>
-        <v>4.49</v>
+        <f>C4 * 3.79</f>
+        <v>3.79</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>61</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1884,13 +1890,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C5" s="7">
         <v>1</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>17</v>
@@ -1908,20 +1914,20 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C6" s="7">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="10">
-        <f>C6 * 1</f>
-        <v>1</v>
+        <f>C6 * 1.59</f>
+        <v>1.59</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>11</v>
@@ -1932,13 +1938,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C7" s="7">
         <v>1</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>17</v>
@@ -1956,13 +1962,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C8" s="7">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>17</v>
@@ -1980,13 +1986,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>17</v>
@@ -1996,7 +2002,7 @@
         <v>3.89</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="J9" s="40" t="s">
         <v>50</v>
@@ -2011,13 +2017,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>17</v>
@@ -2027,7 +2033,7 @@
         <v>1.29</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="J10" s="43"/>
       <c r="K10" s="44"/>
@@ -2040,13 +2046,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>17</v>
@@ -2056,7 +2062,7 @@
         <v>1.77</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="J11" s="43"/>
       <c r="K11" s="44"/>
@@ -2069,13 +2075,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>17</v>
@@ -2085,7 +2091,7 @@
         <v>2.12</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="J12" s="46"/>
       <c r="K12" s="47"/>
@@ -2094,9 +2100,31 @@
       <c r="N12" s="48"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>10</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="7">
+        <v>1</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="10">
+        <f>C13 * 2.15</f>
+        <v>2.15</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>37</v>
+      </c>
       <c r="J13" s="25">
         <f>SUM(F4:F30)</f>
-        <v>21.14</v>
+        <v>23.18</v>
       </c>
       <c r="K13" s="26"/>
       <c r="L13" s="26"/>
@@ -2131,7 +2159,7 @@
     <mergeCell ref="J13:N16"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G12">
+  <conditionalFormatting sqref="G4:G13">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Not ordered"</formula>
     </cfRule>
@@ -2142,8 +2170,8 @@
       <formula>"In Stock"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G12" xr:uid="{5C30DADA-6449-478F-B571-319D09B3C008}">
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G13" xr:uid="{5C30DADA-6449-478F-B571-319D09B3C008}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Deleted Old library, added new library, changed the components using the new library
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\parts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDA4E2D-E441-413A-81B4-54D370246057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5D7A36-C04E-409F-8CE0-6A8D6C22E2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
+    <workbookView xWindow="-21600" yWindow="-9210" windowWidth="21810" windowHeight="15930" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Receiver" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="79">
   <si>
     <t>No.</t>
   </si>
@@ -66,12 +66,6 @@
     <t>USB-C Cable</t>
   </si>
   <si>
-    <t>USB-C Cable 3m</t>
-  </si>
-  <si>
-    <t>https://www.amazon.de/ANMIEL-Typ-C-Kabel-Ladekabel-Datenkabel-geflochten/dp/B09C3HH7KJ/ref=sr_1_6?__mk_de_DE=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=1HUJ8X6PSQNU8&amp;dib=eyJ2IjoiMSJ9.ZH0eL8XvX3DTxCgYcgGTokPY-OCGP9OmCfUbJRX_O8dVp8Y1XLwoEsrPFcvnPVLZvmFR-zCeVbO2opkI9v6wstHb3PzAZOQLPOyeihnSe59NsRuwoXQmF8VlHnoIDHRuSmQaxgReVVoqtUnIHtv6TfrKTgO9Kh6iiAGngLh5Ulc8iYjsqR6B1GuoUGYiygCZirhfQUZHJkvbFNL__RF-xSf5BIU2C9X4cmz_-YjN3Lo.3DULeIhGb1u3SODSffwhRyhMYPrRy90LZrRDQ7fSg-g&amp;dib_tag=se&amp;keywords=usb%2Bc%2Bkabel%2Bdata%2B3m&amp;qid=1761953154&amp;sprefix=usb%2Bc%2Bkabel%2Bdata%2B3m%2Caps%2C103&amp;sr=8-6&amp;th=1</t>
-  </si>
-  <si>
     <t>Not ordered</t>
   </si>
   <si>
@@ -135,9 +129,6 @@
     <t>Cer. Capacitors</t>
   </si>
   <si>
-    <t>300 teile/los 50 V 2PF-0,1 UF 30</t>
-  </si>
-  <si>
     <t>Gravi Tax Marble Run</t>
   </si>
   <si>
@@ -277,6 +268,12 @@
   </si>
   <si>
     <t>Infrarot Reflektierende Sensor IR 4x</t>
+  </si>
+  <si>
+    <t>In stock</t>
+  </si>
+  <si>
+    <t>300 teile/los 50 V 2PF-0,1 UF 30 THT</t>
   </si>
 </sst>
 </file>
@@ -638,7 +635,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -693,9 +690,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -708,6 +702,12 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -779,12 +779,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1164,7 +1158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5785CA-F4AE-4464-AE2C-5F7A426F62CB}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.42578125" customWidth="1"/>
@@ -1175,26 +1169,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="36"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="37"/>
       <c r="J1" s="19"/>
       <c r="K1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="37"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="A2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="40"/>
       <c r="J2" s="19"/>
       <c r="K2" s="19"/>
     </row>
@@ -1212,7 +1206,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>6</v>
@@ -1226,7 +1220,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -1235,546 +1229,543 @@
         <v>5</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F4" s="10">
         <v>4.49</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
+        <f>A4 + 1</f>
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F5" s="10">
         <f>C5 * 3.69</f>
         <v>7.38</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+      <c r="A6" s="1">
+        <f t="shared" ref="A6:A24" si="0">A5 + 1</f>
         <v>3</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="16">
-        <v>1</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="18">
-        <v>8.15</v>
+      <c r="C6" s="7">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="10">
+        <v>1.89</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C7" s="7">
         <v>1</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F7" s="10">
-        <v>1.89</v>
+        <f>C7 * 8.29</f>
+        <v>8.2899999999999991</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F8" s="10">
-        <f>C8 * 8.29</f>
-        <v>8.2899999999999991</v>
+        <f>C8 * 2.47</f>
+        <v>4.9400000000000004</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="7">
-        <v>2</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="B9" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="16">
+        <v>1</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="18">
+        <v>250</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J9" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="42"/>
+      <c r="L9" s="42"/>
+      <c r="M9" s="42"/>
+      <c r="N9" s="43"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="10">
-        <f>C9 * 2.47</f>
-        <v>4.9400000000000004</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J9" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
-      <c r="N9" s="42"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
-        <v>7</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>13</v>
-      </c>
       <c r="C10" s="16">
         <v>1</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="18">
-        <v>250</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F10" s="18"/>
       <c r="G10" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J10" s="43"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="45"/>
+        <v>9</v>
+      </c>
+      <c r="J10" s="44"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="46"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="1">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B11" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="16">
-        <v>1</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="18"/>
+      <c r="B11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="7">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="10">
+        <v>16.989999999999998</v>
+      </c>
       <c r="G11" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J11" s="43"/>
-      <c r="K11" s="44"/>
-      <c r="L11" s="44"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="45"/>
+        <v>9</v>
+      </c>
+      <c r="J11" s="44"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="46"/>
     </row>
     <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="C12" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="F12" s="10">
-        <v>16.989999999999998</v>
+        <f>C12 * 2.89</f>
+        <v>5.78</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J12" s="46"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="48"/>
+        <v>77</v>
+      </c>
+      <c r="J12" s="47"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="48"/>
+      <c r="M12" s="48"/>
+      <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C13" s="7">
-        <v>2</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>55</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F13" s="10">
-        <f>C13 * 2.89</f>
-        <v>5.78</v>
+        <v>9.5500000000000007</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J13" s="25">
-        <f>SUM(F4:F51)</f>
-        <v>448.42000000000007</v>
-      </c>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="27"/>
+        <v>34</v>
+      </c>
+      <c r="J13" s="26">
+        <f>SUM(F4:F50)</f>
+        <v>440.2700000000001</v>
+      </c>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="28"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C14" s="7">
         <v>1</v>
       </c>
-      <c r="D14" s="14" t="s">
-        <v>58</v>
+      <c r="D14" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="F14" s="10">
-        <v>9.5500000000000007</v>
+        <v>1.35</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J14" s="28"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="29"/>
-      <c r="M14" s="29"/>
-      <c r="N14" s="30"/>
+        <v>34</v>
+      </c>
+      <c r="J14" s="29"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
+      <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C15" s="7">
         <v>1</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F15" s="10">
-        <v>1.35</v>
+        <v>3.69</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J15" s="28"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="30"/>
+        <v>34</v>
+      </c>
+      <c r="J15" s="29"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C16" s="7">
         <v>1</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F16" s="10">
-        <v>3.69</v>
+        <v>1.94</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J16" s="31"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="33"/>
+        <v>77</v>
+      </c>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="34"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="7">
         <v>1</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>29</v>
+      <c r="D17" s="14" t="s">
+        <v>78</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F17" s="10">
-        <v>1.94</v>
+        <v>1.69</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C18" s="7">
         <v>1</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F18" s="10">
-        <v>1.69</v>
+        <v>1.99</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="7">
-        <v>1</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="13" t="s">
+      <c r="B19" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="20">
+        <v>1</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="23">
+        <v>35.99</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="F19" s="10">
-        <v>1.99</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="20">
-        <v>17</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="21">
-        <v>1</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" s="24">
-        <v>35.99</v>
+      <c r="B20" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="20">
+        <v>1</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="F20" s="23">
+        <v>19.79</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="20">
+      <c r="A21" s="1">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B21" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="21">
-        <v>1</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="24">
-        <v>19.79</v>
+      <c r="B21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="7">
+        <v>1</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="10">
+        <v>2.4900000000000002</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C22" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F22" s="10">
-        <v>2.4900000000000002</v>
+        <f>C22 * 1.19</f>
+        <v>3.57</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C23" s="7">
         <v>3</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F23" s="10">
-        <f>C23 * 1.19</f>
-        <v>3.57</v>
+        <f>C23 * 1.49</f>
+        <v>4.47</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="7">
+        <v>1</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="7">
-        <v>3</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>17</v>
-      </c>
       <c r="F24" s="10">
-        <f>C24 * 1.49</f>
-        <v>4.47</v>
+        <f>C24 * 53.99</f>
+        <v>53.99</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>22</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" s="7">
-        <v>1</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="F25" s="10">
-        <f>C25 * 53.99</f>
-        <v>53.99</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1784,7 +1775,7 @@
     <mergeCell ref="J9:N12"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G25">
+  <conditionalFormatting sqref="G4:G24">
     <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Not ordered"</formula>
     </cfRule>
@@ -1796,12 +1787,12 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G25" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G24" xr:uid="{69404353-99F0-41F3-8F9D-7E5C48143DF8}">
       <formula1>"In stock,Ordered,Not ordered"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E12" r:id="rId1" xr:uid="{E8A5AAF1-A457-44FF-B03E-B13CD56D10C7}"/>
+    <hyperlink ref="E11" r:id="rId1" xr:uid="{E8A5AAF1-A457-44FF-B03E-B13CD56D10C7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -1824,26 +1815,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="36"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="37"/>
       <c r="J1" s="19"/>
       <c r="K1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="37"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="A2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="40"/>
       <c r="J2" s="19"/>
       <c r="K2" s="19"/>
     </row>
@@ -1861,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>6</v>
@@ -1875,23 +1866,23 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F4" s="10">
         <f>C4 * 3.79</f>
         <v>3.79</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1899,23 +1890,23 @@
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C5" s="7">
         <v>1</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F5" s="10">
         <f>C5 * 2.3</f>
         <v>2.2999999999999998</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -1923,23 +1914,23 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C6" s="7">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F6" s="10">
         <f>C6 * 1.59</f>
         <v>1.59</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -1947,23 +1938,23 @@
         <v>4</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C7" s="16">
         <v>1</v>
       </c>
-      <c r="D7" s="49" t="s">
-        <v>62</v>
-      </c>
-      <c r="E7" s="50" t="s">
-        <v>17</v>
+      <c r="D7" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>15</v>
       </c>
       <c r="F7" s="18">
         <f>C7 * 2.13</f>
         <v>2.13</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1971,23 +1962,23 @@
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C8" s="7">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F8" s="10">
         <f>C8 * 2.15</f>
         <v>2.15</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -1995,171 +1986,171 @@
         <v>6</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9" s="10">
         <f>C9 * 3.89</f>
         <v>3.89</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J9" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
-      <c r="N9" s="42"/>
+        <v>34</v>
+      </c>
+      <c r="J9" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="42"/>
+      <c r="L9" s="42"/>
+      <c r="M9" s="42"/>
+      <c r="N9" s="43"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>7</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F10" s="10">
         <f>C10 * 1.29</f>
         <v>1.29</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J10" s="43"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="45"/>
+        <v>34</v>
+      </c>
+      <c r="J10" s="44"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="46"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>8</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F11" s="10">
         <f>C11 * 1.77</f>
         <v>1.77</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J11" s="43"/>
-      <c r="K11" s="44"/>
-      <c r="L11" s="44"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="45"/>
+        <v>34</v>
+      </c>
+      <c r="J11" s="44"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="46"/>
     </row>
     <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>9</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F12" s="10">
         <f>C12 * 2.12</f>
         <v>2.12</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J12" s="46"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="48"/>
+        <v>34</v>
+      </c>
+      <c r="J12" s="47"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="48"/>
+      <c r="M12" s="48"/>
+      <c r="N12" s="49"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>10</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C13" s="7">
         <v>1</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F13" s="10">
         <f>C13 * 2.15</f>
         <v>2.15</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J13" s="25">
+        <v>34</v>
+      </c>
+      <c r="J13" s="26">
         <f>SUM(F4:F30)</f>
         <v>23.18</v>
       </c>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="28"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J14" s="28"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="29"/>
-      <c r="M14" s="29"/>
-      <c r="N14" s="30"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
+      <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J15" s="28"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="30"/>
+      <c r="J15" s="29"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="31"/>
     </row>
     <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="J16" s="31"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="33"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Finished withmaster screen schematic
</commit_message>
<xml_diff>
--- a/parts/Marble-Station-Part-List.xlsx
+++ b/parts/Marble-Station-Part-List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\parts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5D7A36-C04E-409F-8CE0-6A8D6C22E2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA3408E-DDEE-4368-8046-19043322DD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21600" yWindow="-9210" windowWidth="21810" windowHeight="15930" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
+    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{C4091438-3C34-46B4-BEF6-AD84959AFF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Receiver" sheetId="1" r:id="rId1"/>
@@ -1235,7 +1235,7 @@
         <v>4.49</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1507,7 +1507,7 @@
         <v>1.35</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="J14" s="29"/>
       <c r="K14" s="30"/>
@@ -1618,7 +1618,7 @@
         <v>1.99</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1715,7 +1715,7 @@
         <v>3.57</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1978,7 +1978,7 @@
         <v>2.15</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>